<commit_message>
Changing residual embedment calculation method and some troubleshooting on the UD method weighting calcs
</commit_message>
<xml_diff>
--- a/PSI_inputs.xlsx
+++ b/PSI_inputs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AUSM504495\Documents\GitHub\WSP_PSI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46EF4DD2-A6BA-4306-8931-6CC90821D682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{801A3DAD-0E1F-4C50-AD35-1A962725E203}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1D4F1EAD-D63C-4463-81B7-10D96C3C5F00}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="112">
   <si>
     <t>Input File for Pipe-Soil Interaction Analysis</t>
   </si>
@@ -326,12 +326,6 @@
   </si>
   <si>
     <t>Automated Fit</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
-    <t>LN</t>
   </si>
   <si>
     <t>Min Value</t>
@@ -770,7 +764,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
@@ -785,7 +779,7 @@
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
@@ -835,7 +829,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17A463C4-1722-4182-9BE8-8462E138567F}">
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
@@ -894,7 +888,7 @@
         <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -910,7 +904,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B7">
         <v>60</v>
@@ -919,7 +913,7 @@
         <v>80</v>
       </c>
       <c r="G7" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -936,7 +930,7 @@
         <v>10</v>
       </c>
       <c r="G8" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -952,7 +946,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B10">
         <v>60</v>
@@ -961,7 +955,7 @@
         <v>80</v>
       </c>
       <c r="G10" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -969,10 +963,10 @@
         <v>86</v>
       </c>
       <c r="B11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G11" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1039,7 +1033,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>82</v>
       </c>
@@ -1050,12 +1044,12 @@
         <v>83</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>92</v>
       </c>
@@ -1069,14 +1063,14 @@
         <v>77</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>30</v>
       </c>
       <c r="G20" s="1"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -1093,11 +1087,11 @@
       <c r="F21" t="s">
         <v>72</v>
       </c>
-      <c r="H21" t="s">
+      <c r="G21" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>73</v>
       </c>
@@ -1114,11 +1108,11 @@
       <c r="F22" t="s">
         <v>72</v>
       </c>
-      <c r="H22" t="s">
+      <c r="G22" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -1135,11 +1129,11 @@
       <c r="F23" t="s">
         <v>72</v>
       </c>
-      <c r="H23" t="s">
+      <c r="G23" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -1156,11 +1150,11 @@
       <c r="F24" t="s">
         <v>72</v>
       </c>
-      <c r="H24" t="s">
+      <c r="G24" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>24</v>
       </c>
@@ -1180,13 +1174,10 @@
         <v>95</v>
       </c>
       <c r="G25" t="s">
-        <v>96</v>
-      </c>
-      <c r="H25" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -1203,11 +1194,11 @@
       <c r="F26" t="s">
         <v>72</v>
       </c>
-      <c r="H26" t="s">
+      <c r="G26" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>93</v>
       </c>
@@ -1223,11 +1214,11 @@
       <c r="F27" t="s">
         <v>72</v>
       </c>
-      <c r="H27" t="s">
+      <c r="G27" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>26</v>
       </c>
@@ -1247,13 +1238,10 @@
         <v>95</v>
       </c>
       <c r="G28" t="s">
-        <v>97</v>
-      </c>
-      <c r="H28" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>27</v>
       </c>
@@ -1271,11 +1259,11 @@
       <c r="F29" t="s">
         <v>72</v>
       </c>
-      <c r="H29" t="s">
+      <c r="G29" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>28</v>
       </c>
@@ -1293,11 +1281,11 @@
       <c r="F30" t="s">
         <v>72</v>
       </c>
-      <c r="H30" t="s">
+      <c r="G30" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>29</v>
       </c>
@@ -1314,11 +1302,11 @@
       <c r="F31" t="s">
         <v>72</v>
       </c>
-      <c r="H31" t="s">
+      <c r="G31" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>42</v>
       </c>
@@ -1338,13 +1326,10 @@
         <v>95</v>
       </c>
       <c r="G32" t="s">
-        <v>97</v>
-      </c>
-      <c r="H32" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>44</v>
       </c>
@@ -1364,13 +1349,10 @@
         <v>95</v>
       </c>
       <c r="G33" t="s">
-        <v>97</v>
-      </c>
-      <c r="H33" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>70</v>
       </c>
@@ -1390,13 +1372,10 @@
         <v>95</v>
       </c>
       <c r="G34" t="s">
-        <v>97</v>
-      </c>
-      <c r="H34" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>45</v>
       </c>
@@ -1416,13 +1395,10 @@
         <v>95</v>
       </c>
       <c r="G35" t="s">
-        <v>97</v>
-      </c>
-      <c r="H35" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>46</v>
       </c>
@@ -1439,22 +1415,22 @@
       <c r="F36" t="s">
         <v>72</v>
       </c>
-      <c r="H36" t="s">
+      <c r="G36" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>47</v>
       </c>
       <c r="B37" s="3">
+        <v>1</v>
+      </c>
+      <c r="C37" s="3">
         <v>1.5</v>
       </c>
-      <c r="C37" s="3">
-        <v>4.33</v>
-      </c>
       <c r="D37" s="3">
-        <v>8.33</v>
+        <v>2</v>
       </c>
       <c r="E37" s="3">
         <v>1</v>
@@ -1463,13 +1439,10 @@
         <v>95</v>
       </c>
       <c r="G37" t="s">
-        <v>97</v>
-      </c>
-      <c r="H37" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>48</v>
       </c>
@@ -1489,13 +1462,10 @@
         <v>95</v>
       </c>
       <c r="G38" t="s">
-        <v>97</v>
-      </c>
-      <c r="H38" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>49</v>
       </c>
@@ -1515,13 +1485,10 @@
         <v>95</v>
       </c>
       <c r="G39" t="s">
-        <v>96</v>
-      </c>
-      <c r="H39" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>50</v>
       </c>
@@ -1538,11 +1505,11 @@
       <c r="F40" t="s">
         <v>72</v>
       </c>
-      <c r="H40" t="s">
+      <c r="G40" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>51</v>
       </c>
@@ -1559,11 +1526,11 @@
       <c r="F41" t="s">
         <v>72</v>
       </c>
-      <c r="H41" t="s">
+      <c r="G41" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>52</v>
       </c>
@@ -1580,11 +1547,11 @@
       <c r="F42" t="s">
         <v>72</v>
       </c>
-      <c r="H42" t="s">
+      <c r="G42" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>53</v>
       </c>
@@ -1604,13 +1571,10 @@
         <v>95</v>
       </c>
       <c r="G43" t="s">
-        <v>97</v>
-      </c>
-      <c r="H43" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>54</v>
       </c>
@@ -1630,13 +1594,10 @@
         <v>95</v>
       </c>
       <c r="G44" t="s">
-        <v>96</v>
-      </c>
-      <c r="H44" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>55</v>
       </c>
@@ -1653,11 +1614,11 @@
       <c r="F45" t="s">
         <v>72</v>
       </c>
-      <c r="H45" t="s">
+      <c r="G45" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>88</v>
       </c>
@@ -1677,13 +1638,10 @@
         <v>95</v>
       </c>
       <c r="G46" t="s">
-        <v>96</v>
-      </c>
-      <c r="H46" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
     </row>
@@ -1727,13 +1685,13 @@
         <v>92</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1866,7 +1824,7 @@
         <v>42</v>
       </c>
       <c r="C14" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D14">
         <f t="shared" si="0"/>
@@ -1882,7 +1840,7 @@
         <v>42</v>
       </c>
       <c r="C15" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D15">
         <f t="shared" si="0"/>
@@ -1898,7 +1856,7 @@
         <v>42</v>
       </c>
       <c r="C16" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D16">
         <f t="shared" si="0"/>
@@ -1914,7 +1872,7 @@
         <v>42</v>
       </c>
       <c r="C17" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D17">
         <f t="shared" si="0"/>
@@ -1930,7 +1888,7 @@
         <v>42</v>
       </c>
       <c r="C18" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D18">
         <f t="shared" si="0"/>
@@ -1956,7 +1914,7 @@
         <v>42</v>
       </c>
       <c r="C20" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D20">
         <f t="shared" si="0"/>
@@ -2002,7 +1960,7 @@
         <v>42</v>
       </c>
       <c r="C24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D24">
         <f t="shared" si="0"/>
@@ -2018,7 +1976,7 @@
         <v>42</v>
       </c>
       <c r="C25" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D25">
         <f t="shared" si="0"/>
@@ -2044,7 +2002,7 @@
         <v>42</v>
       </c>
       <c r="C27" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D27">
         <f t="shared" si="0"/>

</xml_diff>

<commit_message>
Changes to weighting to account for where different methods are more reliable, and addition of model factor to the post-processing for figures and 5, 50, 95% (note saved data is without model factor so it isn't accidentally applied repeatedly
</commit_message>
<xml_diff>
--- a/PSI_inputs.xlsx
+++ b/PSI_inputs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AUSM504495\Documents\GitHub\WSP_PSI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{801A3DAD-0E1F-4C50-AD35-1A962725E203}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{241122DD-720E-4608-BB35-981DD12D3EA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1D4F1EAD-D63C-4463-81B7-10D96C3C5F00}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="114">
   <si>
     <t>Input File for Pipe-Soil Interaction Analysis</t>
   </si>
@@ -374,6 +374,12 @@
   </si>
   <si>
     <t>% Min and Max weighting applied to Generalised FE Lat_res result if used in conjunction with another Lat_res Model; applied based on embedment and where accuracy of other models is expected to be lower</t>
+  </si>
+  <si>
+    <t>Model_fct</t>
+  </si>
+  <si>
+    <t>% factor applied to all results to arbitrarily account for additional uncertainty by increaisng the bounds; applied linearly for each result where min/1.2 and max*1.2; MEAN WILL BE AFFECTED UNLESS IT IS HALF-WAY BETWEEN MIN AND MAX IN MAGNITUDE</t>
   </si>
 </sst>
 </file>
@@ -829,7 +835,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17A463C4-1722-4182-9BE8-8462E138567F}">
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
@@ -1044,303 +1050,291 @@
         <v>83</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>33</v>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>112</v>
+      </c>
+      <c r="B18">
+        <v>1.2</v>
+      </c>
+      <c r="G18" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B21" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C21" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D21" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="E21" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="F21" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="G20" s="1"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>21</v>
-      </c>
-      <c r="B21" s="2">
-        <v>0.32990000000000003</v>
-      </c>
-      <c r="C21" s="2">
-        <v>0.32990000000000003</v>
-      </c>
-      <c r="D21" s="2">
-        <v>0.32990000000000003</v>
-      </c>
-      <c r="E21" s="2"/>
-      <c r="F21" t="s">
-        <v>72</v>
-      </c>
-      <c r="G21" t="s">
-        <v>75</v>
-      </c>
+      <c r="G21" s="1"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>73</v>
+        <v>21</v>
       </c>
       <c r="B22" s="2">
-        <v>2.6599999999999999E-2</v>
+        <v>0.32990000000000003</v>
       </c>
       <c r="C22" s="2">
-        <v>2.6599999999999999E-2</v>
+        <v>0.32990000000000003</v>
       </c>
       <c r="D22" s="2">
-        <v>2.6599999999999999E-2</v>
+        <v>0.32990000000000003</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" t="s">
         <v>72</v>
       </c>
       <c r="G22" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>22</v>
+        <v>73</v>
       </c>
       <c r="B23" s="2">
-        <v>0.89749999999999996</v>
+        <v>2.6599999999999999E-2</v>
       </c>
       <c r="C23" s="2">
-        <v>0.89749999999999996</v>
+        <v>2.6599999999999999E-2</v>
       </c>
       <c r="D23" s="2">
-        <v>0.89749999999999996</v>
+        <v>2.6599999999999999E-2</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s">
         <v>72</v>
       </c>
       <c r="G23" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B24" s="2">
-        <v>1.5022</v>
+        <v>0.89749999999999996</v>
       </c>
       <c r="C24" s="2">
-        <v>1.5022</v>
+        <v>0.89749999999999996</v>
       </c>
       <c r="D24" s="2">
-        <v>1.5022</v>
+        <v>0.89749999999999996</v>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" t="s">
         <v>72</v>
       </c>
       <c r="G24" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B25" s="2">
-        <v>0.95650000000000002</v>
+        <v>1.5022</v>
       </c>
       <c r="C25" s="2">
-        <v>1.0155000000000001</v>
+        <v>1.5022</v>
       </c>
       <c r="D25" s="2">
-        <v>1.0745</v>
-      </c>
-      <c r="E25" s="2">
-        <v>0.89749999999999996</v>
-      </c>
+        <v>1.5022</v>
+      </c>
+      <c r="E25" s="2"/>
       <c r="F25" t="s">
-        <v>95</v>
+        <v>72</v>
       </c>
       <c r="G25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>25</v>
-      </c>
-      <c r="B26" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="C26" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="D26" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="E26" s="4"/>
+        <v>24</v>
+      </c>
+      <c r="B26" s="2">
+        <v>0.95650000000000002</v>
+      </c>
+      <c r="C26" s="2">
+        <v>1.0155000000000001</v>
+      </c>
+      <c r="D26" s="2">
+        <v>1.0745</v>
+      </c>
+      <c r="E26" s="2">
+        <v>0.89749999999999996</v>
+      </c>
       <c r="F26" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
       <c r="G26" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>93</v>
-      </c>
-      <c r="B27">
-        <v>61675</v>
-      </c>
-      <c r="C27">
-        <v>61675</v>
-      </c>
-      <c r="D27">
-        <v>61675</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="B27" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="C27" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="D27" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="E27" s="4"/>
       <c r="F27" t="s">
         <v>72</v>
       </c>
       <c r="G27" t="s">
-        <v>94</v>
+        <v>37</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>26</v>
+        <v>93</v>
       </c>
       <c r="B28">
-        <v>27</v>
+        <v>61675</v>
       </c>
       <c r="C28">
-        <v>100</v>
+        <v>61675</v>
       </c>
       <c r="D28">
-        <v>236</v>
-      </c>
-      <c r="E28">
-        <v>10</v>
+        <v>61675</v>
       </c>
       <c r="F28" t="s">
-        <v>95</v>
+        <v>72</v>
       </c>
       <c r="G28" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>26</v>
+      </c>
+      <c r="B29">
         <v>27</v>
       </c>
-      <c r="B29" s="2">
+      <c r="C29">
+        <v>100</v>
+      </c>
+      <c r="D29">
+        <v>236</v>
+      </c>
+      <c r="E29">
+        <v>10</v>
+      </c>
+      <c r="F29" t="s">
+        <v>95</v>
+      </c>
+      <c r="G29" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>27</v>
+      </c>
+      <c r="B30" s="2">
         <f>1/12</f>
         <v>8.3333333333333329E-2</v>
       </c>
-      <c r="C29" s="2">
+      <c r="C30" s="2">
         <v>8.3333333333333329E-2</v>
       </c>
-      <c r="D29" s="2">
+      <c r="D30" s="2">
         <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="E29" s="2"/>
-      <c r="F29" t="s">
-        <v>72</v>
-      </c>
-      <c r="G29" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>28</v>
-      </c>
-      <c r="B30" s="2">
-        <f>1/24</f>
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C30" s="2">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="D30" s="2">
-        <v>4.1666666666666664E-2</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" t="s">
         <v>72</v>
       </c>
       <c r="G30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B31" s="2">
-        <v>8.3333333333333329E-2</v>
+        <f>1/24</f>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="C31" s="2">
-        <v>8.3333333333333329E-2</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="D31" s="2">
-        <v>8.3333333333333329E-2</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s">
         <v>72</v>
       </c>
       <c r="G31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>42</v>
-      </c>
-      <c r="B32" s="3">
-        <v>0</v>
-      </c>
-      <c r="C32" s="3">
-        <v>0.35</v>
-      </c>
-      <c r="D32" s="3">
-        <v>3.57</v>
-      </c>
-      <c r="E32" s="3">
-        <v>0</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="B32" s="2">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="C32" s="2">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="D32" s="2">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E32" s="2"/>
       <c r="F32" t="s">
-        <v>95</v>
+        <v>72</v>
       </c>
       <c r="G32" t="s">
-        <v>57</v>
+        <v>40</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B33" s="3">
-        <v>1.33</v>
+        <v>0</v>
       </c>
       <c r="C33" s="3">
-        <v>4.84</v>
+        <v>0.35</v>
       </c>
       <c r="D33" s="3">
-        <v>14.29</v>
+        <v>3.57</v>
       </c>
       <c r="E33" s="3">
         <v>0</v>
@@ -1349,21 +1343,21 @@
         <v>95</v>
       </c>
       <c r="G33" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>70</v>
+        <v>44</v>
       </c>
       <c r="B34" s="3">
         <v>1.33</v>
       </c>
       <c r="C34" s="3">
-        <v>3</v>
+        <v>4.84</v>
       </c>
       <c r="D34" s="3">
-        <v>7.72</v>
+        <v>14.29</v>
       </c>
       <c r="E34" s="3">
         <v>0</v>
@@ -1372,111 +1366,111 @@
         <v>95</v>
       </c>
       <c r="G34" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="B35" s="3">
-        <v>3.04</v>
+        <v>1.33</v>
       </c>
       <c r="C35" s="3">
-        <v>4.2</v>
+        <v>3</v>
       </c>
       <c r="D35" s="3">
-        <v>6.96</v>
+        <v>7.72</v>
       </c>
       <c r="E35" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F35" t="s">
         <v>95</v>
       </c>
       <c r="G35" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B36" s="3">
-        <v>3</v>
+        <v>3.04</v>
       </c>
       <c r="C36" s="3">
-        <v>5</v>
+        <v>4.2</v>
       </c>
       <c r="D36" s="3">
-        <v>7</v>
-      </c>
-      <c r="E36" s="3"/>
+        <v>6.96</v>
+      </c>
+      <c r="E36" s="3">
+        <v>1</v>
+      </c>
       <c r="F36" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
       <c r="G36" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B37" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C37" s="3">
-        <v>1.5</v>
+        <v>5</v>
       </c>
       <c r="D37" s="3">
-        <v>2</v>
-      </c>
-      <c r="E37" s="3">
-        <v>1</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="E37" s="3"/>
       <c r="F37" t="s">
-        <v>95</v>
+        <v>72</v>
       </c>
       <c r="G37" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>48</v>
-      </c>
-      <c r="B38">
-        <v>0.44</v>
-      </c>
-      <c r="C38">
-        <v>17.73</v>
-      </c>
-      <c r="D38">
-        <v>503.82</v>
+        <v>47</v>
+      </c>
+      <c r="B38" s="3">
+        <v>1</v>
+      </c>
+      <c r="C38" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="D38" s="3">
+        <v>2</v>
       </c>
       <c r="E38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F38" t="s">
         <v>95</v>
       </c>
       <c r="G38" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>49</v>
-      </c>
-      <c r="B39" s="4">
-        <v>0.22</v>
-      </c>
-      <c r="C39" s="4">
-        <v>0.28499999999999998</v>
-      </c>
-      <c r="D39" s="4">
-        <v>0.35</v>
+        <v>48</v>
+      </c>
+      <c r="B39">
+        <v>0.44</v>
+      </c>
+      <c r="C39">
+        <v>17.73</v>
+      </c>
+      <c r="D39">
+        <v>503.82</v>
       </c>
       <c r="E39" s="3">
         <v>0</v>
@@ -1485,54 +1479,56 @@
         <v>95</v>
       </c>
       <c r="G39" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B40" s="4">
-        <v>0.4</v>
+        <v>0.22</v>
       </c>
       <c r="C40" s="4">
-        <v>0.4</v>
+        <v>0.28499999999999998</v>
       </c>
       <c r="D40" s="4">
-        <v>0.4</v>
-      </c>
-      <c r="E40" s="4"/>
+        <v>0.35</v>
+      </c>
+      <c r="E40" s="3">
+        <v>0</v>
+      </c>
       <c r="F40" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
       <c r="G40" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B41" s="4">
-        <v>2</v>
+        <v>0.4</v>
       </c>
       <c r="C41" s="4">
-        <v>2.25</v>
+        <v>0.4</v>
       </c>
       <c r="D41" s="4">
-        <v>2.5</v>
+        <v>0.4</v>
       </c>
       <c r="E41" s="4"/>
       <c r="F41" t="s">
         <v>72</v>
       </c>
       <c r="G41" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B42" s="4">
         <v>2</v>
@@ -1548,44 +1544,42 @@
         <v>72</v>
       </c>
       <c r="G42" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>53</v>
-      </c>
-      <c r="B43">
-        <v>24</v>
-      </c>
-      <c r="C43">
-        <v>30</v>
-      </c>
-      <c r="D43">
-        <v>42</v>
-      </c>
-      <c r="E43" s="3">
-        <v>0</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="B43" s="4">
+        <v>2</v>
+      </c>
+      <c r="C43" s="4">
+        <v>2.25</v>
+      </c>
+      <c r="D43" s="4">
+        <v>2.5</v>
+      </c>
+      <c r="E43" s="4"/>
       <c r="F43" t="s">
-        <v>95</v>
+        <v>72</v>
       </c>
       <c r="G43" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>54</v>
-      </c>
-      <c r="B44" s="4">
-        <v>0.22</v>
-      </c>
-      <c r="C44" s="4">
-        <v>0.28499999999999998</v>
-      </c>
-      <c r="D44" s="4">
-        <v>0.35</v>
+        <v>53</v>
+      </c>
+      <c r="B44">
+        <v>24</v>
+      </c>
+      <c r="C44">
+        <v>30</v>
+      </c>
+      <c r="D44">
+        <v>42</v>
       </c>
       <c r="E44" s="3">
         <v>0</v>
@@ -1594,56 +1588,79 @@
         <v>95</v>
       </c>
       <c r="G44" t="s">
-        <v>91</v>
+        <v>68</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B45" s="4">
-        <v>0.4</v>
+        <v>0.22</v>
       </c>
       <c r="C45" s="4">
-        <v>0.4</v>
+        <v>0.28499999999999998</v>
       </c>
       <c r="D45" s="4">
-        <v>0.4</v>
-      </c>
-      <c r="E45" s="4"/>
+        <v>0.35</v>
+      </c>
+      <c r="E45" s="3">
+        <v>0</v>
+      </c>
       <c r="F45" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
       <c r="G45" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>55</v>
+      </c>
+      <c r="B46" s="4">
+        <v>0.4</v>
+      </c>
+      <c r="C46" s="4">
+        <v>0.4</v>
+      </c>
+      <c r="D46" s="4">
+        <v>0.4</v>
+      </c>
+      <c r="E46" s="4"/>
+      <c r="F46" t="s">
+        <v>72</v>
+      </c>
+      <c r="G46" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>88</v>
       </c>
-      <c r="B46" s="3">
+      <c r="B47" s="3">
         <v>26.6</v>
       </c>
-      <c r="C46" s="3">
+      <c r="C47" s="3">
         <v>34.6</v>
       </c>
-      <c r="D46" s="4">
+      <c r="D47" s="4">
         <v>41.3</v>
       </c>
-      <c r="E46" s="3">
+      <c r="E47" s="3">
         <v>0</v>
       </c>
-      <c r="F46" t="s">
+      <c r="F47" t="s">
         <v>95</v>
       </c>
-      <c r="G46" t="s">
+      <c r="G47" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B47" s="3"/>
-      <c r="C47" s="3"/>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B48" s="3"/>
+      <c r="C48" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1655,7 +1672,7 @@
           <x14:formula1>
             <xm:f>Intro!$A$13:$A$19</xm:f>
           </x14:formula1>
-          <xm:sqref>F21:F46</xm:sqref>
+          <xm:sqref>F22:F47</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4A6C1404-CBB2-46E4-A208-B5A1886B394C}">
           <x14:formula1>
@@ -1696,7 +1713,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="str">
-        <f>Inputs!A21</f>
+        <f>Inputs!A22</f>
         <v>D</v>
       </c>
       <c r="D2" t="str">
@@ -1706,7 +1723,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
-        <f>Inputs!A22</f>
+        <f>Inputs!A23</f>
         <v>t</v>
       </c>
       <c r="D3" t="str">
@@ -1716,7 +1733,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="str">
-        <f>Inputs!A23</f>
+        <f>Inputs!A24</f>
         <v>W_empty</v>
       </c>
       <c r="D4" t="str">
@@ -1726,7 +1743,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
-        <f>Inputs!A24</f>
+        <f>Inputs!A25</f>
         <v>W_hydro</v>
       </c>
       <c r="D5" t="str">
@@ -1736,7 +1753,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
-        <f>Inputs!A25</f>
+        <f>Inputs!A26</f>
         <v>W_op</v>
       </c>
       <c r="D6" t="str">
@@ -1746,7 +1763,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
-        <f>Inputs!A26</f>
+        <f>Inputs!A27</f>
         <v>alpha</v>
       </c>
       <c r="D7" t="str">
@@ -1756,7 +1773,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
-        <f>Inputs!A27</f>
+        <f>Inputs!A28</f>
         <v>EI</v>
       </c>
       <c r="D8" t="str">
@@ -1766,7 +1783,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="str">
-        <f>Inputs!A28</f>
+        <f>Inputs!A29</f>
         <v>T0</v>
       </c>
       <c r="D9" t="str">
@@ -1776,7 +1793,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="str">
-        <f>Inputs!A29</f>
+        <f>Inputs!A30</f>
         <v>t_aslaid</v>
       </c>
       <c r="D10" t="str">
@@ -1786,7 +1803,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="str">
-        <f>Inputs!A30</f>
+        <f>Inputs!A31</f>
         <v>t_hydro</v>
       </c>
       <c r="D11" t="str">
@@ -1796,7 +1813,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="str">
-        <f>Inputs!A31</f>
+        <f>Inputs!A32</f>
         <v>t_preop</v>
       </c>
       <c r="D12" t="str">
@@ -1806,7 +1823,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="str">
-        <f>Inputs!A32</f>
+        <f>Inputs!A33</f>
         <v>su_mudline</v>
       </c>
       <c r="D13" t="str">
@@ -1817,7 +1834,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="str">
-        <f>Inputs!A33</f>
+        <f>Inputs!A34</f>
         <v>su_inv</v>
       </c>
       <c r="B14" t="s">
@@ -1833,7 +1850,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="str">
-        <f>Inputs!A34</f>
+        <f>Inputs!A35</f>
         <v>delta_su</v>
       </c>
       <c r="B15" t="s">
@@ -1849,7 +1866,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="str">
-        <f>Inputs!A35</f>
+        <f>Inputs!A36</f>
         <v>gamma_sub</v>
       </c>
       <c r="B16" t="s">
@@ -1865,7 +1882,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="str">
-        <f>Inputs!A36</f>
+        <f>Inputs!A37</f>
         <v>pipelay_St</v>
       </c>
       <c r="B17" t="s">
@@ -1881,7 +1898,7 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="str">
-        <f>Inputs!A37</f>
+        <f>Inputs!A38</f>
         <v>lateral_St</v>
       </c>
       <c r="B18" t="s">
@@ -1897,7 +1914,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="str">
-        <f>Inputs!A38</f>
+        <f>Inputs!A39</f>
         <v>cv</v>
       </c>
       <c r="D19" t="str">
@@ -1907,7 +1924,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="str">
-        <f>Inputs!A39</f>
+        <f>Inputs!A40</f>
         <v>SHANSEP_S</v>
       </c>
       <c r="B20" t="s">
@@ -1923,7 +1940,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="str">
-        <f>Inputs!A40</f>
+        <f>Inputs!A41</f>
         <v>SHANSEP_m</v>
       </c>
       <c r="D21" t="str">
@@ -1933,7 +1950,7 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="str">
-        <f>Inputs!A41</f>
+        <f>Inputs!A42</f>
         <v>ka</v>
       </c>
       <c r="D22" t="str">
@@ -1943,7 +1960,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="str">
-        <f>Inputs!A42</f>
+        <f>Inputs!A43</f>
         <v>kp</v>
       </c>
       <c r="D23" t="str">
@@ -1953,7 +1970,7 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="str">
-        <f>Inputs!A43</f>
+        <f>Inputs!A44</f>
         <v>phi</v>
       </c>
       <c r="B24" t="s">
@@ -1969,7 +1986,7 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="str">
-        <f>Inputs!A44</f>
+        <f>Inputs!A45</f>
         <v>int_SHANSEP_S</v>
       </c>
       <c r="B25" t="s">
@@ -1985,7 +2002,7 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="str">
-        <f>Inputs!A45</f>
+        <f>Inputs!A46</f>
         <v>int_SHANSEP_m</v>
       </c>
       <c r="D26" t="str">
@@ -1995,7 +2012,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="str">
-        <f>Inputs!A46</f>
+        <f>Inputs!A47</f>
         <v>delta</v>
       </c>
       <c r="B27" t="s">

</xml_diff>

<commit_message>
Adding cyclic transition from UD to D method
</commit_message>
<xml_diff>
--- a/PSI_inputs.xlsx
+++ b/PSI_inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AUSM504495\Documents\GitHub\WSP_PSI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{241122DD-720E-4608-BB35-981DD12D3EA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{167ACBE4-8D7D-4316-A3DE-9760D256A2A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1D4F1EAD-D63C-4463-81B7-10D96C3C5F00}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1D4F1EAD-D63C-4463-81B7-10D96C3C5F00}"/>
   </bookViews>
   <sheets>
     <sheet name="Intro" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="116">
   <si>
     <t>Input File for Pipe-Soil Interaction Analysis</t>
   </si>
@@ -70,9 +70,6 @@
     <t>Ax_model</t>
   </si>
   <si>
-    <t>Lat_cyc_model</t>
-  </si>
-  <si>
     <t>No_cycles</t>
   </si>
   <si>
@@ -94,9 +91,6 @@
     <t>% undrained: SAFEBUCK with rate effects from DNVGL-RP-F114 = 0 (SAFEBUCK chosen over DNV as it directly uses interface strength profile rather than applying alpha factor for roughness and epsilon factor for partial remoulding, but otherwise calculation is the same), drained: DNVGL-RP-F114/SAFEBUCK = 10</t>
   </si>
   <si>
-    <t>% undrained: SAFEBUCK = 0 (not included in DNVGL-RP-F114)</t>
-  </si>
-  <si>
     <t>% number of cycles to model for lateral cyclic resistance calculations</t>
   </si>
   <si>
@@ -380,6 +374,18 @@
   </si>
   <si>
     <t>% factor applied to all results to arbitrarily account for additional uncertainty by increaisng the bounds; applied linearly for each result where min/1.2 and max*1.2; MEAN WILL BE AFFECTED UNLESS IT IS HALF-WAY BETWEEN MIN AND MAX IN MAGNITUDE</t>
+  </si>
+  <si>
+    <t>N50</t>
+  </si>
+  <si>
+    <t>% number of cycles for 50% transition between UD and D; Yan et al. 2014 examples approx. N50 = 2 (N95 = 5) and N50 = 4 (N95 = 18); more examples shown in excel 'Cyclic Curves from Yan 2014'</t>
+  </si>
+  <si>
+    <t>Cyc_model</t>
+  </si>
+  <si>
+    <t>% SAFEBUCK UD Lateral = 0 (not included in DNVGL-RP-F114, no axial option included); White &amp; Cheuk 2008 = 1;  Internal method transitioning from UD to D = 2</t>
   </si>
 </sst>
 </file>
@@ -770,7 +776,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
@@ -785,47 +791,47 @@
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -835,7 +841,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17A463C4-1722-4182-9BE8-8462E138567F}">
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
@@ -844,18 +850,18 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B2">
         <v>10000</v>
       </c>
       <c r="G2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -866,7 +872,7 @@
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -877,7 +883,7 @@
         <v>0</v>
       </c>
       <c r="G4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -894,7 +900,7 @@
         <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -905,12 +911,12 @@
         <v>0</v>
       </c>
       <c r="G6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B7">
         <v>60</v>
@@ -919,7 +925,7 @@
         <v>80</v>
       </c>
       <c r="G7" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -936,23 +942,23 @@
         <v>10</v>
       </c>
       <c r="G8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B9">
         <v>0</v>
       </c>
       <c r="G9" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B10">
         <v>60</v>
@@ -961,18 +967,18 @@
         <v>80</v>
       </c>
       <c r="G10" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B11">
         <v>2</v>
       </c>
       <c r="G11" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -986,23 +992,23 @@
         <v>10</v>
       </c>
       <c r="G12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>114</v>
       </c>
       <c r="B13">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G13" t="s">
-        <v>18</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B14">
         <v>1</v>
@@ -1014,542 +1020,532 @@
         <v>100</v>
       </c>
       <c r="G14" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>112</v>
       </c>
       <c r="B15">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G15" t="s">
-        <v>56</v>
+        <v>113</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B16">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G16" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>82</v>
-      </c>
-      <c r="B17" t="s">
-        <v>95</v>
+        <v>41</v>
+      </c>
+      <c r="B17">
+        <v>0.5</v>
       </c>
       <c r="G17" t="s">
-        <v>83</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>112</v>
-      </c>
-      <c r="B18">
+        <v>80</v>
+      </c>
+      <c r="B18" t="s">
+        <v>93</v>
+      </c>
+      <c r="G18" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>110</v>
+      </c>
+      <c r="B19">
         <v>1.2</v>
       </c>
-      <c r="G18" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>33</v>
+      <c r="G19" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="G21" s="1"/>
+        <v>31</v>
+      </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>21</v>
-      </c>
-      <c r="B22" s="2">
-        <v>0.32990000000000003</v>
-      </c>
-      <c r="C22" s="2">
-        <v>0.32990000000000003</v>
-      </c>
-      <c r="D22" s="2">
-        <v>0.32990000000000003</v>
-      </c>
-      <c r="E22" s="2"/>
-      <c r="F22" t="s">
-        <v>72</v>
-      </c>
-      <c r="G22" t="s">
+      <c r="A22" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="1" t="s">
         <v>75</v>
       </c>
+      <c r="E22" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G22" s="1"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>19</v>
       </c>
       <c r="B23" s="2">
-        <v>2.6599999999999999E-2</v>
+        <v>0.32990000000000003</v>
       </c>
       <c r="C23" s="2">
-        <v>2.6599999999999999E-2</v>
+        <v>0.32990000000000003</v>
       </c>
       <c r="D23" s="2">
-        <v>2.6599999999999999E-2</v>
+        <v>0.32990000000000003</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G23" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>71</v>
       </c>
       <c r="B24" s="2">
-        <v>0.89749999999999996</v>
+        <v>2.6599999999999999E-2</v>
       </c>
       <c r="C24" s="2">
-        <v>0.89749999999999996</v>
+        <v>2.6599999999999999E-2</v>
       </c>
       <c r="D24" s="2">
-        <v>0.89749999999999996</v>
+        <v>2.6599999999999999E-2</v>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" t="s">
+        <v>70</v>
+      </c>
+      <c r="G24" t="s">
         <v>72</v>
-      </c>
-      <c r="G24" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B25" s="2">
-        <v>1.5022</v>
+        <v>0.89749999999999996</v>
       </c>
       <c r="C25" s="2">
-        <v>1.5022</v>
+        <v>0.89749999999999996</v>
       </c>
       <c r="D25" s="2">
-        <v>1.5022</v>
+        <v>0.89749999999999996</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G25" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B26" s="2">
-        <v>0.95650000000000002</v>
+        <v>1.5022</v>
       </c>
       <c r="C26" s="2">
-        <v>1.0155000000000001</v>
+        <v>1.5022</v>
       </c>
       <c r="D26" s="2">
-        <v>1.0745</v>
-      </c>
-      <c r="E26" s="2">
-        <v>0.89749999999999996</v>
-      </c>
+        <v>1.5022</v>
+      </c>
+      <c r="E26" s="2"/>
       <c r="F26" t="s">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="G26" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>25</v>
-      </c>
-      <c r="B27" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="C27" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="D27" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="E27" s="4"/>
+        <v>22</v>
+      </c>
+      <c r="B27" s="2">
+        <v>0.95650000000000002</v>
+      </c>
+      <c r="C27" s="2">
+        <v>1.0155000000000001</v>
+      </c>
+      <c r="D27" s="2">
+        <v>1.0745</v>
+      </c>
+      <c r="E27" s="2">
+        <v>0.89749999999999996</v>
+      </c>
       <c r="F27" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="G27" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>93</v>
-      </c>
-      <c r="B28">
-        <v>61675</v>
-      </c>
-      <c r="C28">
-        <v>61675</v>
-      </c>
-      <c r="D28">
-        <v>61675</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="B28" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="C28" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="D28" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="E28" s="4"/>
       <c r="F28" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G28" t="s">
-        <v>94</v>
+        <v>35</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>26</v>
+        <v>91</v>
       </c>
       <c r="B29">
-        <v>27</v>
+        <v>61675</v>
       </c>
       <c r="C29">
-        <v>100</v>
+        <v>61675</v>
       </c>
       <c r="D29">
-        <v>236</v>
-      </c>
-      <c r="E29">
-        <v>10</v>
+        <v>61675</v>
       </c>
       <c r="F29" t="s">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="G29" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>24</v>
+      </c>
+      <c r="B30">
         <v>27</v>
       </c>
-      <c r="B30" s="2">
+      <c r="C30">
+        <v>100</v>
+      </c>
+      <c r="D30">
+        <v>236</v>
+      </c>
+      <c r="E30">
+        <v>10</v>
+      </c>
+      <c r="F30" t="s">
+        <v>93</v>
+      </c>
+      <c r="G30" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>25</v>
+      </c>
+      <c r="B31" s="2">
         <f>1/12</f>
         <v>8.3333333333333329E-2</v>
       </c>
-      <c r="C30" s="2">
+      <c r="C31" s="2">
         <v>8.3333333333333329E-2</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D31" s="2">
         <v>8.3333333333333329E-2</v>
       </c>
-      <c r="E30" s="2"/>
-      <c r="F30" t="s">
-        <v>72</v>
-      </c>
-      <c r="G30" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>28</v>
-      </c>
-      <c r="B31" s="2">
+      <c r="E31" s="2"/>
+      <c r="F31" t="s">
+        <v>70</v>
+      </c>
+      <c r="G31" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>26</v>
+      </c>
+      <c r="B32" s="2">
         <f>1/24</f>
         <v>4.1666666666666664E-2</v>
       </c>
-      <c r="C31" s="2">
+      <c r="C32" s="2">
         <v>4.1666666666666664E-2</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D32" s="2">
         <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="E31" s="2"/>
-      <c r="F31" t="s">
-        <v>72</v>
-      </c>
-      <c r="G31" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>29</v>
-      </c>
-      <c r="B32" s="2">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="C32" s="2">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="D32" s="2">
-        <v>8.3333333333333329E-2</v>
       </c>
       <c r="E32" s="2"/>
       <c r="F32" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G32" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>42</v>
-      </c>
-      <c r="B33" s="3">
-        <v>0</v>
-      </c>
-      <c r="C33" s="3">
-        <v>0.35</v>
-      </c>
-      <c r="D33" s="3">
-        <v>3.57</v>
-      </c>
-      <c r="E33" s="3">
-        <v>0</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="B33" s="2">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="C33" s="2">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="D33" s="2">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E33" s="2"/>
       <c r="F33" t="s">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="G33" t="s">
-        <v>57</v>
+        <v>38</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B34" s="3">
-        <v>1.33</v>
+        <v>0</v>
       </c>
       <c r="C34" s="3">
-        <v>4.84</v>
+        <v>0.35</v>
       </c>
       <c r="D34" s="3">
-        <v>14.29</v>
+        <v>3.57</v>
       </c>
       <c r="E34" s="3">
         <v>0</v>
       </c>
       <c r="F34" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="G34" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="B35" s="3">
         <v>1.33</v>
       </c>
       <c r="C35" s="3">
-        <v>3</v>
+        <v>4.84</v>
       </c>
       <c r="D35" s="3">
-        <v>7.72</v>
+        <v>14.29</v>
       </c>
       <c r="E35" s="3">
         <v>0</v>
       </c>
       <c r="F35" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="G35" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>45</v>
+        <v>68</v>
       </c>
       <c r="B36" s="3">
-        <v>3.04</v>
+        <v>1.33</v>
       </c>
       <c r="C36" s="3">
-        <v>4.2</v>
+        <v>3</v>
       </c>
       <c r="D36" s="3">
-        <v>6.96</v>
+        <v>7.72</v>
       </c>
       <c r="E36" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F36" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="G36" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B37" s="3">
-        <v>3</v>
+        <v>3.04</v>
       </c>
       <c r="C37" s="3">
-        <v>5</v>
+        <v>4.2</v>
       </c>
       <c r="D37" s="3">
-        <v>7</v>
-      </c>
-      <c r="E37" s="3"/>
+        <v>6.96</v>
+      </c>
+      <c r="E37" s="3">
+        <v>1</v>
+      </c>
       <c r="F37" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="G37" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B38" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C38" s="3">
-        <v>1.5</v>
+        <v>5</v>
       </c>
       <c r="D38" s="3">
-        <v>2</v>
-      </c>
-      <c r="E38" s="3">
-        <v>1</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="E38" s="3"/>
       <c r="F38" t="s">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="G38" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>48</v>
-      </c>
-      <c r="B39">
-        <v>0.44</v>
-      </c>
-      <c r="C39">
-        <v>17.73</v>
-      </c>
-      <c r="D39">
-        <v>503.82</v>
+        <v>45</v>
+      </c>
+      <c r="B39" s="3">
+        <v>1</v>
+      </c>
+      <c r="C39" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="D39" s="3">
+        <v>2</v>
       </c>
       <c r="E39" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F39" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="G39" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>49</v>
-      </c>
-      <c r="B40" s="4">
-        <v>0.22</v>
-      </c>
-      <c r="C40" s="4">
-        <v>0.28499999999999998</v>
-      </c>
-      <c r="D40" s="4">
-        <v>0.35</v>
+        <v>46</v>
+      </c>
+      <c r="B40">
+        <v>0.44</v>
+      </c>
+      <c r="C40">
+        <v>17.73</v>
+      </c>
+      <c r="D40">
+        <v>503.82</v>
       </c>
       <c r="E40" s="3">
         <v>0</v>
       </c>
       <c r="F40" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="G40" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B41" s="4">
-        <v>0.4</v>
+        <v>0.22</v>
       </c>
       <c r="C41" s="4">
-        <v>0.4</v>
+        <v>0.28499999999999998</v>
       </c>
       <c r="D41" s="4">
-        <v>0.4</v>
-      </c>
-      <c r="E41" s="4"/>
+        <v>0.35</v>
+      </c>
+      <c r="E41" s="3">
+        <v>0</v>
+      </c>
       <c r="F41" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="G41" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B42" s="4">
-        <v>2</v>
+        <v>0.4</v>
       </c>
       <c r="C42" s="4">
-        <v>2.25</v>
+        <v>0.4</v>
       </c>
       <c r="D42" s="4">
-        <v>2.5</v>
+        <v>0.4</v>
       </c>
       <c r="E42" s="4"/>
       <c r="F42" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G42" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B43" s="4">
         <v>2</v>
@@ -1562,105 +1558,126 @@
       </c>
       <c r="E43" s="4"/>
       <c r="F43" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G43" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>53</v>
-      </c>
-      <c r="B44">
-        <v>24</v>
-      </c>
-      <c r="C44">
-        <v>30</v>
-      </c>
-      <c r="D44">
-        <v>42</v>
-      </c>
-      <c r="E44" s="3">
-        <v>0</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="B44" s="4">
+        <v>2</v>
+      </c>
+      <c r="C44" s="4">
+        <v>2.25</v>
+      </c>
+      <c r="D44" s="4">
+        <v>2.5</v>
+      </c>
+      <c r="E44" s="4"/>
       <c r="F44" t="s">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="G44" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>54</v>
-      </c>
-      <c r="B45" s="4">
-        <v>0.22</v>
-      </c>
-      <c r="C45" s="4">
-        <v>0.28499999999999998</v>
-      </c>
-      <c r="D45" s="4">
-        <v>0.35</v>
+        <v>51</v>
+      </c>
+      <c r="B45">
+        <v>24</v>
+      </c>
+      <c r="C45">
+        <v>30</v>
+      </c>
+      <c r="D45">
+        <v>42</v>
       </c>
       <c r="E45" s="3">
         <v>0</v>
       </c>
       <c r="F45" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="G45" t="s">
-        <v>91</v>
+        <v>66</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B46" s="4">
-        <v>0.4</v>
+        <v>0.22</v>
       </c>
       <c r="C46" s="4">
-        <v>0.4</v>
+        <v>0.28499999999999998</v>
       </c>
       <c r="D46" s="4">
-        <v>0.4</v>
-      </c>
-      <c r="E46" s="4"/>
+        <v>0.35</v>
+      </c>
+      <c r="E46" s="3">
+        <v>0</v>
+      </c>
       <c r="F46" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="G46" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
+        <v>53</v>
+      </c>
+      <c r="B47" s="4">
+        <v>0.4</v>
+      </c>
+      <c r="C47" s="4">
+        <v>0.4</v>
+      </c>
+      <c r="D47" s="4">
+        <v>0.4</v>
+      </c>
+      <c r="E47" s="4"/>
+      <c r="F47" t="s">
+        <v>70</v>
+      </c>
+      <c r="G47" t="s">
         <v>88</v>
       </c>
-      <c r="B47" s="3">
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>86</v>
+      </c>
+      <c r="B48" s="3">
         <v>26.6</v>
       </c>
-      <c r="C47" s="3">
+      <c r="C48" s="3">
         <v>34.6</v>
       </c>
-      <c r="D47" s="4">
+      <c r="D48" s="4">
         <v>41.3</v>
       </c>
-      <c r="E47" s="3">
+      <c r="E48" s="3">
         <v>0</v>
       </c>
-      <c r="F47" t="s">
-        <v>95</v>
-      </c>
-      <c r="G47" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B48" s="3"/>
-      <c r="C48" s="3"/>
+      <c r="F48" t="s">
+        <v>93</v>
+      </c>
+      <c r="G48" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B49" s="3"/>
+      <c r="C49" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1672,13 +1689,13 @@
           <x14:formula1>
             <xm:f>Intro!$A$13:$A$19</xm:f>
           </x14:formula1>
-          <xm:sqref>F22:F47</xm:sqref>
+          <xm:sqref>F23:F48</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4A6C1404-CBB2-46E4-A208-B5A1886B394C}">
           <x14:formula1>
             <xm:f>Intro!$A$14:$A$19</xm:f>
           </x14:formula1>
-          <xm:sqref>B17</xm:sqref>
+          <xm:sqref>B18</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1699,21 +1716,21 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="str">
-        <f>Inputs!A22</f>
+        <f>Inputs!A23</f>
         <v>D</v>
       </c>
       <c r="D2" t="str">
@@ -1723,7 +1740,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
-        <f>Inputs!A23</f>
+        <f>Inputs!A24</f>
         <v>t</v>
       </c>
       <c r="D3" t="str">
@@ -1733,7 +1750,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="str">
-        <f>Inputs!A24</f>
+        <f>Inputs!A25</f>
         <v>W_empty</v>
       </c>
       <c r="D4" t="str">
@@ -1743,7 +1760,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
-        <f>Inputs!A25</f>
+        <f>Inputs!A26</f>
         <v>W_hydro</v>
       </c>
       <c r="D5" t="str">
@@ -1753,7 +1770,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
-        <f>Inputs!A26</f>
+        <f>Inputs!A27</f>
         <v>W_op</v>
       </c>
       <c r="D6" t="str">
@@ -1763,7 +1780,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
-        <f>Inputs!A27</f>
+        <f>Inputs!A28</f>
         <v>alpha</v>
       </c>
       <c r="D7" t="str">
@@ -1773,7 +1790,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
-        <f>Inputs!A28</f>
+        <f>Inputs!A29</f>
         <v>EI</v>
       </c>
       <c r="D8" t="str">
@@ -1783,7 +1800,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="str">
-        <f>Inputs!A29</f>
+        <f>Inputs!A30</f>
         <v>T0</v>
       </c>
       <c r="D9" t="str">
@@ -1793,7 +1810,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="str">
-        <f>Inputs!A30</f>
+        <f>Inputs!A31</f>
         <v>t_aslaid</v>
       </c>
       <c r="D10" t="str">
@@ -1803,7 +1820,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="str">
-        <f>Inputs!A31</f>
+        <f>Inputs!A32</f>
         <v>t_hydro</v>
       </c>
       <c r="D11" t="str">
@@ -1813,7 +1830,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="str">
-        <f>Inputs!A32</f>
+        <f>Inputs!A33</f>
         <v>t_preop</v>
       </c>
       <c r="D12" t="str">
@@ -1823,7 +1840,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="str">
-        <f>Inputs!A33</f>
+        <f>Inputs!A34</f>
         <v>su_mudline</v>
       </c>
       <c r="D13" t="str">
@@ -1834,14 +1851,14 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="str">
-        <f>Inputs!A34</f>
+        <f>Inputs!A35</f>
         <v>su_inv</v>
       </c>
       <c r="B14" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C14" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D14">
         <f t="shared" si="0"/>
@@ -1850,14 +1867,14 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="str">
-        <f>Inputs!A35</f>
+        <f>Inputs!A36</f>
         <v>delta_su</v>
       </c>
       <c r="B15" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C15" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D15">
         <f t="shared" si="0"/>
@@ -1866,14 +1883,14 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="str">
-        <f>Inputs!A36</f>
+        <f>Inputs!A37</f>
         <v>gamma_sub</v>
       </c>
       <c r="B16" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C16" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D16">
         <f t="shared" si="0"/>
@@ -1882,14 +1899,14 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="str">
-        <f>Inputs!A37</f>
+        <f>Inputs!A38</f>
         <v>pipelay_St</v>
       </c>
       <c r="B17" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C17" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D17">
         <f t="shared" si="0"/>
@@ -1898,14 +1915,14 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="str">
-        <f>Inputs!A38</f>
+        <f>Inputs!A39</f>
         <v>lateral_St</v>
       </c>
       <c r="B18" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C18" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D18">
         <f t="shared" si="0"/>
@@ -1914,7 +1931,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="str">
-        <f>Inputs!A39</f>
+        <f>Inputs!A40</f>
         <v>cv</v>
       </c>
       <c r="D19" t="str">
@@ -1924,14 +1941,14 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="str">
-        <f>Inputs!A40</f>
+        <f>Inputs!A41</f>
         <v>SHANSEP_S</v>
       </c>
       <c r="B20" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C20" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D20">
         <f t="shared" si="0"/>
@@ -1940,7 +1957,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="str">
-        <f>Inputs!A41</f>
+        <f>Inputs!A42</f>
         <v>SHANSEP_m</v>
       </c>
       <c r="D21" t="str">
@@ -1950,7 +1967,7 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="str">
-        <f>Inputs!A42</f>
+        <f>Inputs!A43</f>
         <v>ka</v>
       </c>
       <c r="D22" t="str">
@@ -1960,7 +1977,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="str">
-        <f>Inputs!A43</f>
+        <f>Inputs!A44</f>
         <v>kp</v>
       </c>
       <c r="D23" t="str">
@@ -1970,14 +1987,14 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="str">
-        <f>Inputs!A44</f>
+        <f>Inputs!A45</f>
         <v>phi</v>
       </c>
       <c r="B24" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C24" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D24">
         <f t="shared" si="0"/>
@@ -1986,14 +2003,14 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="str">
-        <f>Inputs!A45</f>
+        <f>Inputs!A46</f>
         <v>int_SHANSEP_S</v>
       </c>
       <c r="B25" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C25" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D25">
         <f t="shared" si="0"/>
@@ -2002,7 +2019,7 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="str">
-        <f>Inputs!A46</f>
+        <f>Inputs!A47</f>
         <v>int_SHANSEP_m</v>
       </c>
       <c r="D26" t="str">
@@ -2012,14 +2029,14 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="str">
-        <f>Inputs!A47</f>
+        <f>Inputs!A48</f>
         <v>delta</v>
       </c>
       <c r="B27" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C27" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D27">
         <f t="shared" si="0"/>

</xml_diff>